<commit_message>
Fixing some bugs with personnel, tables
</commit_message>
<xml_diff>
--- a/MetadataTemplate.xlsx
+++ b/MetadataTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://doimspp-my.sharepoint.com/personal/kherrmann_nps_gov/Documents/Desktop/Code/RStudio/GitHub/MetadataOuroboros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1055" documentId="8_{2F8795CF-CDDF-43BA-97D9-07A87AE2952A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BF155DC-223E-47AA-82F8-A6069B8E4F06}"/>
+  <xr:revisionPtr revIDLastSave="1057" documentId="8_{2F8795CF-CDDF-43BA-97D9-07A87AE2952A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3006F33C-9663-4E1F-B561-3E573163F72C}"/>
   <bookViews>
-    <workbookView xWindow="132" yWindow="732" windowWidth="22908" windowHeight="12222" firstSheet="4" activeTab="9" xr2:uid="{F3CFC82C-CDFA-43A3-931A-18FF91478685}"/>
+    <workbookView xWindow="132" yWindow="2178" windowWidth="22908" windowHeight="12222" firstSheet="4" activeTab="9" xr2:uid="{F3CFC82C-CDFA-43A3-931A-18FF91478685}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="12" r:id="rId1"/>
@@ -4286,7 +4286,7 @@
     <cellStyle name="Input" xfId="1" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="66">
+  <dxfs count="42">
     <dxf>
       <fill>
         <patternFill>
@@ -4548,25 +4548,15 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i/>
+      </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFFF99"/>
+          <bgColor theme="3" tint="0.749961851863155"/>
         </patternFill>
       </fill>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <fill>
@@ -4646,38 +4636,6 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
         </patternFill>
       </fill>
       <border>
@@ -4882,184 +4840,6 @@
       <fill>
         <patternFill>
           <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="3" tint="0.749961851863155"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF99"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5442,7 +5222,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45618FF2-10A0-4111-8C15-36F09A916DBC}">
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="25.15625" customWidth="1"/>
@@ -5598,88 +5378,112 @@
       <c r="I6" s="35"/>
       <c r="J6" s="35"/>
     </row>
-    <row r="10" spans="1:10" ht="72.900000000000006" x14ac:dyDescent="0.7">
-      <c r="A10" s="8" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="47"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="35"/>
+      <c r="J7" s="35"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="47"/>
+      <c r="B8" s="47"/>
+      <c r="C8" s="47"/>
+      <c r="D8" s="47"/>
+      <c r="E8" s="47"/>
+      <c r="F8" s="47"/>
+      <c r="G8" s="47"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="35"/>
+    </row>
+    <row r="12" spans="1:10" ht="72.900000000000006" x14ac:dyDescent="0.7">
+      <c r="A12" s="8" t="s">
         <v>1085</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="9" t="s">
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="53" t="s">
+      <c r="G12" s="53" t="s">
         <v>1100</v>
       </c>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9" t="s">
+      <c r="H12" s="9"/>
+      <c r="I12" s="9" t="s">
         <v>1082</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="J12" s="9" t="s">
         <v>1082</v>
       </c>
     </row>
-    <row r="11" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="4" t="s">
+    <row r="13" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H13" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I13" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="J13" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="G12" t="s">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="G14" t="s">
         <v>32</v>
       </c>
-      <c r="H12"/>
-      <c r="I12" s="35"/>
-      <c r="J12" s="35"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.55000000000000004">
-      <c r="G13" t="s">
+      <c r="H14"/>
+      <c r="I14" s="35"/>
+      <c r="J14" s="35"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.55000000000000004">
+      <c r="G15" t="s">
         <v>30</v>
       </c>
-      <c r="H13"/>
-      <c r="I13" s="35"/>
-      <c r="J13" s="35"/>
+      <c r="H15"/>
+      <c r="I15" s="35"/>
+      <c r="J15" s="35"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:J1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A12:H13">
+  <conditionalFormatting sqref="A14:H15">
     <cfRule type="expression" dxfId="7" priority="2">
-      <formula>A12=""</formula>
+      <formula>A14=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B14:H120">
+  <conditionalFormatting sqref="B16:H122">
     <cfRule type="expression" dxfId="6" priority="1">
-      <formula>AND($A14&lt;&gt;"", B14="")</formula>
+      <formula>AND($A16&lt;&gt;"", B16="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1">
@@ -14127,90 +13931,81 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" formatCells="0"/>
-  <conditionalFormatting sqref="D7:J8 C4:C254 A7:B8 A9:J1048576 A1:J1 A5:J6 H3:J4 A2:F4 I2:J2">
-    <cfRule type="expression" dxfId="43" priority="10">
+  <conditionalFormatting sqref="A1:J1 A2:F4 A5:J6 D7:J8 A9:J1048576 H3:J4 C4:C254 A7:B8">
+    <cfRule type="expression" dxfId="41" priority="10">
       <formula>$B1="attributeName"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C4:C1048576">
-    <cfRule type="expression" dxfId="42" priority="20">
+    <cfRule type="expression" dxfId="40" priority="20">
       <formula>AND($C4="",$B4&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8">
-    <cfRule type="expression" dxfId="41" priority="22">
+    <cfRule type="expression" dxfId="39" priority="22">
       <formula>$B7="attributeName"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="24">
+    <cfRule type="expression" dxfId="38" priority="24">
       <formula>AND($C8="",$B7&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:D2 E1:E1048576">
-    <cfRule type="expression" dxfId="39" priority="9">
+  <conditionalFormatting sqref="E1:E1048576 C2:D2">
+    <cfRule type="expression" dxfId="37" priority="9">
       <formula>$E1="!Add units here!"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1:F1048576">
-    <cfRule type="expression" dxfId="38" priority="18">
+    <cfRule type="expression" dxfId="36" priority="18">
       <formula>$F1="!Add datetime specifier here!"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2">
-    <cfRule type="expression" dxfId="37" priority="8">
+  <conditionalFormatting sqref="F2:H2">
+    <cfRule type="expression" dxfId="35" priority="2">
       <formula>$E2="!Add units here!"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G1 G5:G1048576">
-    <cfRule type="expression" dxfId="36" priority="11">
+    <cfRule type="expression" dxfId="34" priority="11">
       <formula>AND($H1="NA",$B1&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="13">
+    <cfRule type="expression" dxfId="33" priority="13">
       <formula>$B1&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G2">
+    <cfRule type="expression" dxfId="32" priority="1">
+      <formula>AND($H2="",$B2&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="31" priority="4">
+      <formula>AND($H2="NA",$B2&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="30" priority="5">
+      <formula>$B2&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3">
+    <cfRule type="expression" dxfId="29" priority="27">
+      <formula>$B4="attributeName"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="28" priority="33">
+      <formula>AND($H4="NA",$B4&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="27" priority="34">
+      <formula>$B4&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:J2">
+    <cfRule type="expression" dxfId="26" priority="3">
+      <formula>$B2="attributeName"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H1 H3:H1048576">
-    <cfRule type="expression" dxfId="34" priority="15">
+    <cfRule type="expression" dxfId="25" priority="15">
       <formula>AND($H1="",$B1&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3">
-    <cfRule type="expression" dxfId="32" priority="27">
-      <formula>$B4="attributeName"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G3">
-    <cfRule type="expression" dxfId="31" priority="33">
-      <formula>AND($H4="NA",$B4&lt;&gt;"")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="30" priority="34">
-      <formula>$B4&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:H2">
-    <cfRule type="expression" dxfId="29" priority="3">
-      <formula>$B2="attributeName"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2">
-    <cfRule type="expression" dxfId="28" priority="4">
-      <formula>AND($H2="NA",$B2&lt;&gt;"")</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="27" priority="5">
-      <formula>$B2&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H2">
-    <cfRule type="expression" dxfId="26" priority="6">
-      <formula>AND($H2="",$B2&lt;&gt;"")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:H2">
-    <cfRule type="expression" dxfId="25" priority="2">
-      <formula>$E2="!Add units here!"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2">
-    <cfRule type="expression" dxfId="24" priority="1">
+    <cfRule type="expression" dxfId="24" priority="6">
       <formula>AND($H2="",$B2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>